<commit_message>
Add raw header fixture 1-row-horizontal-merge (B–C merged).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_header/test_cases.xlsx
+++ b/excel/testdata/raw_header/test_cases.xlsx
@@ -10,22 +10,23 @@
     <sheet name="1-row-simple" sheetId="1" r:id="rId1"/>
     <sheet name="1-row-empty-header" sheetId="2" r:id="rId5"/>
     <sheet name="1-row-line-break" sheetId="3" r:id="rId6"/>
-    <sheet name="2-row-simple" sheetId="4" r:id="rId7"/>
-    <sheet name="2-row-empty-cell" sheetId="5" r:id="rId8"/>
-    <sheet name="2-row-horizontal-merge" sheetId="6" r:id="rId9"/>
-    <sheet name="2-row-horizontal-merge-repeated" sheetId="7" r:id="rId10"/>
-    <sheet name="2-row-vertical-merge" sheetId="8" r:id="rId11"/>
-    <sheet name="2-row-vertical-merge-repeated" sheetId="9" r:id="rId12"/>
-    <sheet name="2-row-bidirectional-merge" sheetId="10" r:id="rId13"/>
-    <sheet name="2-row-bidirectional-merge-rep" sheetId="11" r:id="rId14"/>
-    <sheet name="2-row-mixed-merge" sheetId="12" r:id="rId15"/>
+    <sheet name="1-row-horizontal-merge" sheetId="4" r:id="rId7"/>
+    <sheet name="2-row-simple" sheetId="5" r:id="rId8"/>
+    <sheet name="2-row-empty-cell" sheetId="6" r:id="rId9"/>
+    <sheet name="2-row-horizontal-merge" sheetId="7" r:id="rId10"/>
+    <sheet name="2-row-horizontal-merge-repeated" sheetId="8" r:id="rId11"/>
+    <sheet name="2-row-vertical-merge" sheetId="9" r:id="rId12"/>
+    <sheet name="2-row-vertical-merge-repeated" sheetId="10" r:id="rId13"/>
+    <sheet name="2-row-bidirectional-merge" sheetId="11" r:id="rId14"/>
+    <sheet name="2-row-bidirectional-merge-rep" sheetId="12" r:id="rId15"/>
+    <sheet name="2-row-mixed-merge" sheetId="13" r:id="rId16"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>headerA</t>
   </si>
@@ -42,6 +43,12 @@
 line breaks</t>
   </si>
   <si>
+    <t>headerBC</t>
+  </si>
+  <si>
+    <t>headerD</t>
+  </si>
+  <si>
     <t>group1</t>
   </si>
   <si>
@@ -52,9 +59,6 @@
   </si>
   <si>
     <t>group 3</t>
-  </si>
-  <si>
-    <t>headerD</t>
   </si>
   <si>
     <t>headerE</t>
@@ -414,8 +418,43 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>6</v>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -430,7 +469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -442,7 +481,7 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
@@ -450,7 +489,7 @@
         <v>2</v>
       </c>
       <c r="I2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -462,7 +501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -471,45 +510,45 @@
         <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -563,14 +602,63 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>4</v>
       </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
       <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>6</v>
       </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -587,43 +675,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
+      <c r="C1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -644,42 +705,42 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -690,7 +751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -699,10 +760,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -718,39 +779,4 @@
     <mergeCell ref="A1:A2"/>
   </mergeCells>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-  </mergeCells>
-</worksheet>
 </file>
</xml_diff>